<commit_message>
Updates in the transport module
</commit_message>
<xml_diff>
--- a/models/49sectors_exiobase/parameters.xlsx
+++ b/models/49sectors_exiobase/parameters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\01.Feina_CREAF\06.Git_Repos\pymedeas2_vensim\models_for_pymedeas2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{281FE4BF-68F8-4FE1-9473-D6C33D263C08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56E7017E-44B2-417F-93A8-8AFF74DAA9DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="13995" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28050" windowHeight="13995" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Global" sheetId="1" r:id="rId1"/>
@@ -39,33 +39,33 @@
     <definedName name="damage_function_parameter_b" localSheetId="3">Catalonia!#REF!</definedName>
     <definedName name="damage_function_parameter_b" localSheetId="2">Europe!$O$10</definedName>
     <definedName name="damage_function_parameter_b" localSheetId="1">World!$C$28</definedName>
-    <definedName name="employment_factor_biofuels" localSheetId="0">Global!$C$21</definedName>
+    <definedName name="employment_factor_biofuels" localSheetId="0">Global!$C$22</definedName>
     <definedName name="employment_factor_fuel_supply_solids_bioe" localSheetId="0">Global!$E$8</definedName>
-    <definedName name="employment_factors_new_res_elec" localSheetId="0">Global!$C$6:$C$13</definedName>
-    <definedName name="employment_factors_new_res_heat" localSheetId="0">Global!$C$17:$C$19</definedName>
-    <definedName name="employment_factors_o_m_res_elec" localSheetId="0">Global!$D$6:$D$13</definedName>
-    <definedName name="employment_factors_o_m_res_heat" localSheetId="0">Global!$D$17:$D$19</definedName>
-    <definedName name="end_historical_year" localSheetId="0">Global!$C$43</definedName>
-    <definedName name="eol_rr_minerals_alt_techn_res_vs_total_economy" localSheetId="0">Global!$C$23</definedName>
-    <definedName name="gch4_coal" localSheetId="0">Global!$C$37</definedName>
-    <definedName name="gch4_conv_gas" localSheetId="0">Global!$C$35</definedName>
-    <definedName name="gch4_ctl" localSheetId="0">Global!$C$39</definedName>
-    <definedName name="gch4_gtl" localSheetId="0">Global!$C$40</definedName>
-    <definedName name="gch4_oil" localSheetId="0">Global!$C$38</definedName>
-    <definedName name="gch4_unconventional_gas" localSheetId="0">Global!$C$36</definedName>
-    <definedName name="gco2_coal" localSheetId="0">Global!$C$29</definedName>
-    <definedName name="gco2_conventional_gas" localSheetId="0">Global!$C$30</definedName>
-    <definedName name="gco2_conventional_oil" localSheetId="0">Global!$C$31</definedName>
-    <definedName name="gco2_ctl" localSheetId="0">Global!$C$27</definedName>
-    <definedName name="gco2_gtl" localSheetId="0">Global!$C$28</definedName>
-    <definedName name="gco2_shale_oil" localSheetId="0">Global!$C$34</definedName>
-    <definedName name="gco2_unconventional_gas" localSheetId="0">Global!$C$32</definedName>
-    <definedName name="gco2_unconventional_oil" localSheetId="0">Global!$C$33</definedName>
+    <definedName name="employment_factors_new_res_elec" localSheetId="0">Global!$C$6:$C$14</definedName>
+    <definedName name="employment_factors_new_res_heat" localSheetId="0">Global!$C$18:$C$20</definedName>
+    <definedName name="employment_factors_o_m_res_elec" localSheetId="0">Global!$D$6:$D$14</definedName>
+    <definedName name="employment_factors_o_m_res_heat" localSheetId="0">Global!$D$18:$D$20</definedName>
+    <definedName name="end_historical_year" localSheetId="0">Global!$C$44</definedName>
+    <definedName name="eol_rr_minerals_alt_techn_res_vs_total_economy" localSheetId="0">Global!$C$24</definedName>
+    <definedName name="gch4_coal" localSheetId="0">Global!$C$38</definedName>
+    <definedName name="gch4_conv_gas" localSheetId="0">Global!$C$36</definedName>
+    <definedName name="gch4_ctl" localSheetId="0">Global!$C$40</definedName>
+    <definedName name="gch4_gtl" localSheetId="0">Global!$C$41</definedName>
+    <definedName name="gch4_oil" localSheetId="0">Global!$C$39</definedName>
+    <definedName name="gch4_unconventional_gas" localSheetId="0">Global!$C$37</definedName>
+    <definedName name="gco2_coal" localSheetId="0">Global!$C$30</definedName>
+    <definedName name="gco2_conventional_gas" localSheetId="0">Global!$C$31</definedName>
+    <definedName name="gco2_conventional_oil" localSheetId="0">Global!$C$32</definedName>
+    <definedName name="gco2_ctl" localSheetId="0">Global!$C$28</definedName>
+    <definedName name="gco2_gtl" localSheetId="0">Global!$C$29</definedName>
+    <definedName name="gco2_shale_oil" localSheetId="0">Global!$C$35</definedName>
+    <definedName name="gco2_unconventional_gas" localSheetId="0">Global!$C$33</definedName>
+    <definedName name="gco2_unconventional_oil" localSheetId="0">Global!$C$34</definedName>
     <definedName name="global_arable_land" localSheetId="3">Catalonia!#REF!</definedName>
     <definedName name="global_arable_land" localSheetId="2">Europe!$C$9</definedName>
     <definedName name="global_arable_land" localSheetId="1">World!$C$9</definedName>
     <definedName name="historic_population" localSheetId="3">Catalonia!$C$2:$X$2</definedName>
-    <definedName name="historic_population" localSheetId="2">Europe!$C$2:$X$2</definedName>
+    <definedName name="historic_population" localSheetId="2">Europe!$C$2:$AG$2</definedName>
     <definedName name="historic_population" localSheetId="1">World!$C$2:$X$2</definedName>
     <definedName name="initial_population" localSheetId="3">Catalonia!$C$2</definedName>
     <definedName name="initial_population" localSheetId="2">Europe!$C$2</definedName>
@@ -73,12 +73,12 @@
     <definedName name="input_population" localSheetId="3">Catalonia!#REF!</definedName>
     <definedName name="input_population" localSheetId="2">Europe!$C$4:$H$4</definedName>
     <definedName name="input_population" localSheetId="1">World!$C$4:$H$4</definedName>
-    <definedName name="maximum_recycling_rate_minerals" localSheetId="0">Global!$C$24</definedName>
+    <definedName name="maximum_recycling_rate_minerals" localSheetId="0">Global!$C$25</definedName>
     <definedName name="people_relying_on_traditional_biomass" localSheetId="3">Catalonia!$C$5</definedName>
     <definedName name="people_relying_on_traditional_biomass" localSheetId="2">Europe!$C$7</definedName>
     <definedName name="people_relying_on_traditional_biomass" localSheetId="1">World!$C$7</definedName>
-    <definedName name="ratio_total_vs_direct_jobs_res_elec" localSheetId="0">Global!$B$6:$B$13</definedName>
-    <definedName name="ratio_total_vs_direct_jobs_res_heat" localSheetId="0">Global!$B$17:$B$19</definedName>
+    <definedName name="ratio_total_vs_direct_jobs_res_elec" localSheetId="0">Global!$B$6:$B$14</definedName>
+    <definedName name="ratio_total_vs_direct_jobs_res_heat" localSheetId="0">Global!$B$18:$B$20</definedName>
     <definedName name="renewable_water_resources" localSheetId="3">Catalonia!$C$16</definedName>
     <definedName name="renewable_water_resources" localSheetId="2">Europe!$C$21</definedName>
     <definedName name="renewable_water_resources" localSheetId="1">World!$C$21</definedName>
@@ -86,7 +86,7 @@
     <definedName name="time_afforestation" localSheetId="2">Europe!$C$13:$X$13</definedName>
     <definedName name="time_afforestation" localSheetId="1">World!#REF!</definedName>
     <definedName name="time_historic_population" localSheetId="3">Catalonia!$C$1:$X$1</definedName>
-    <definedName name="time_historic_population" localSheetId="2">Europe!$C$1:$X$1</definedName>
+    <definedName name="time_historic_population" localSheetId="2">Europe!$C$1:$AG$1</definedName>
     <definedName name="time_historic_population" localSheetId="1">World!$C$1:$X$1</definedName>
     <definedName name="time_index_projection" localSheetId="3">Catalonia!#REF!</definedName>
     <definedName name="time_index_projection" localSheetId="2">Europe!$C$3:$H$3</definedName>
@@ -325,7 +325,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B19" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000009000000}">
+    <comment ref="B20" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000009000000}">
       <text>
         <r>
           <rPr>
@@ -350,7 +350,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C21" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000A000000}">
+    <comment ref="C22" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000A000000}">
       <text>
         <r>
           <rPr>
@@ -375,7 +375,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C24" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000B000000}">
+    <comment ref="C25" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000B000000}">
       <text>
         <r>
           <rPr>
@@ -400,7 +400,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A27" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000C000000}">
+    <comment ref="A28" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000C000000}">
       <text>
         <r>
           <rPr>
@@ -425,7 +425,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A28" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000D000000}">
+    <comment ref="A29" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000D000000}">
       <text>
         <r>
           <rPr>
@@ -450,7 +450,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A29" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000E000000}">
+    <comment ref="A30" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000E000000}">
       <text>
         <r>
           <rPr>
@@ -475,7 +475,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A30" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000F000000}">
+    <comment ref="A31" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000F000000}">
       <text>
         <r>
           <rPr>
@@ -500,7 +500,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A31" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000010000000}">
+    <comment ref="A32" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000010000000}">
       <text>
         <r>
           <rPr>
@@ -525,7 +525,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A32" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000011000000}">
+    <comment ref="A33" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000011000000}">
       <text>
         <r>
           <rPr>
@@ -551,7 +551,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A33" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000012000000}">
+    <comment ref="A34" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000012000000}">
       <text>
         <r>
           <rPr>
@@ -576,7 +576,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A34" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000013000000}">
+    <comment ref="A35" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000013000000}">
       <text>
         <r>
           <rPr>
@@ -601,7 +601,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A35" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000014000000}">
+    <comment ref="A36" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000014000000}">
       <text>
         <r>
           <rPr>
@@ -626,7 +626,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A36" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000015000000}">
+    <comment ref="A37" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000015000000}">
       <text>
         <r>
           <rPr>
@@ -651,7 +651,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A43" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000016000000}">
+    <comment ref="A44" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000016000000}">
       <text>
         <r>
           <rPr>
@@ -916,7 +916,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C27" authorId="0" shapeId="0" xr:uid="{06DA6D6D-8689-41A5-97B1-E0D7EADE88F8}">
+    <comment ref="C27" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00000B000000}">
       <text>
         <r>
           <rPr>
@@ -966,7 +966,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C28" authorId="0" shapeId="0" xr:uid="{7FF6925C-97DE-40EF-BE7D-E3E1D3948777}">
+    <comment ref="C28" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00000D000000}">
       <text>
         <r>
           <rPr>
@@ -1200,7 +1200,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="89">
   <si>
     <t>Jobs</t>
   </si>
@@ -1464,6 +1464,9 @@
   </si>
   <si>
     <t>We/m2</t>
+  </si>
+  <si>
+    <t>Fuel cell</t>
   </si>
 </sst>
 </file>
@@ -1476,7 +1479,7 @@
     <numFmt numFmtId="166" formatCode="0.00000"/>
     <numFmt numFmtId="167" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -1544,6 +1547,11 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Liberation Sans"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -1577,7 +1585,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -1733,12 +1741,23 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1838,6 +1857,14 @@
     <xf numFmtId="3" fontId="9" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -2232,36 +2259,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:E43"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A2:E44"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="44.7109375" customWidth="1"/>
     <col min="2" max="5" width="14.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B2" s="60" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="60"/>
-      <c r="D2" s="60"/>
-      <c r="E2" s="60"/>
-    </row>
-    <row r="3" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="61" t="s">
+    <row r="2" spans="1:5">
+      <c r="B2" s="64" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="64"/>
+      <c r="D2" s="64"/>
+      <c r="E2" s="64"/>
+    </row>
+    <row r="3" spans="1:5" ht="15" customHeight="1">
+      <c r="B3" s="65" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="62" t="s">
+      <c r="C3" s="66" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D3" s="66"/>
+      <c r="E3" s="66"/>
+    </row>
+    <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="61"/>
+      <c r="B4" s="65"/>
       <c r="C4" s="1" t="s">
         <v>4</v>
       </c>
@@ -2272,7 +2299,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5">
       <c r="A5" s="1"/>
       <c r="B5" s="1" t="s">
         <v>7</v>
@@ -2288,7 +2315,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5">
       <c r="A6" s="2" t="s">
         <v>10</v>
       </c>
@@ -2303,7 +2330,7 @@
       </c>
       <c r="E6" s="5"/>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5">
       <c r="A7" s="6" t="s">
         <v>11</v>
       </c>
@@ -2318,7 +2345,7 @@
       </c>
       <c r="E7" s="5"/>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5">
       <c r="A8" s="6" t="s">
         <v>12</v>
       </c>
@@ -2335,7 +2362,7 @@
         <v>2.9000000000000001E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5">
       <c r="A9" s="6" t="s">
         <v>13</v>
       </c>
@@ -2350,7 +2377,7 @@
       </c>
       <c r="E9" s="5"/>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5">
       <c r="A10" s="6" t="s">
         <v>14</v>
       </c>
@@ -2365,7 +2392,7 @@
       </c>
       <c r="E10" s="5"/>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5">
       <c r="A11" s="6" t="s">
         <v>15</v>
       </c>
@@ -2380,7 +2407,7 @@
       </c>
       <c r="E11" s="5"/>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5">
       <c r="A12" s="6" t="s">
         <v>16</v>
       </c>
@@ -2395,7 +2422,7 @@
       </c>
       <c r="E12" s="5"/>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5">
       <c r="A13" s="6" t="s">
         <v>17</v>
       </c>
@@ -2410,238 +2437,244 @@
       </c>
       <c r="E13" s="5"/>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="7" t="s">
+    <row r="14" spans="1:5">
+      <c r="A14" s="60" t="s">
+        <v>88</v>
+      </c>
+      <c r="B14" s="62">
+        <v>0</v>
+      </c>
+      <c r="C14" s="61">
+        <v>0</v>
+      </c>
+      <c r="D14" s="61">
+        <v>0</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B16" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C16" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="D16" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E15" s="5" t="s">
+      <c r="E16" s="5" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="8"/>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="9" t="s">
+    <row r="17" spans="1:5">
+      <c r="A17" s="8"/>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="B17" s="10">
+      <c r="B18" s="10">
         <v>1</v>
       </c>
-      <c r="C17" s="4">
+      <c r="C18" s="4">
         <v>8.4</v>
       </c>
-      <c r="D17" s="4">
-        <v>0</v>
-      </c>
-      <c r="E17" s="11"/>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="12" t="s">
+      <c r="D18" s="4">
+        <v>0</v>
+      </c>
+      <c r="E18" s="11"/>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B18" s="10">
+      <c r="B19" s="10">
         <v>1.9</v>
       </c>
-      <c r="C18" s="4">
+      <c r="C19" s="4">
         <v>6.9</v>
       </c>
-      <c r="D18" s="4">
-        <v>0</v>
-      </c>
-      <c r="E18" s="11"/>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="12" t="s">
+      <c r="D19" s="4">
+        <v>0</v>
+      </c>
+      <c r="E19" s="11"/>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B19" s="13">
+      <c r="B20" s="13">
         <v>1</v>
       </c>
-      <c r="C19" s="4">
+      <c r="C20" s="4">
         <v>16.899999999999999</v>
       </c>
-      <c r="D19" s="4">
+      <c r="D20" s="4">
         <v>1.5</v>
       </c>
-      <c r="E19" s="14"/>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C20" s="63" t="s">
+      <c r="E20" s="14"/>
+    </row>
+    <row r="21" spans="1:5">
+      <c r="C21" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="D20" s="63"/>
-      <c r="E20" s="15"/>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C21" s="64">
+      <c r="D21" s="67"/>
+      <c r="E21" s="15"/>
+    </row>
+    <row r="22" spans="1:5">
+      <c r="C22" s="68">
         <v>740231.85916702403</v>
       </c>
-      <c r="D21" s="64"/>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="12" t="s">
+      <c r="D22" s="68"/>
+    </row>
+    <row r="24" spans="1:5">
+      <c r="A24" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="B24" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C23" s="17">
+      <c r="C24" s="17">
         <f>1/3</f>
         <v>0.33333333333333331</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="12" t="s">
+    <row r="25" spans="1:5">
+      <c r="A25" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="B25" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C24" s="17">
+      <c r="C25" s="17">
         <v>0.95</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="59" t="s">
+    <row r="27" spans="1:5">
+      <c r="A27" s="63" t="s">
         <v>26</v>
       </c>
-      <c r="B26" s="59"/>
-      <c r="C26" s="59"/>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="6" t="s">
+      <c r="B27" s="63"/>
+      <c r="C27" s="63"/>
+    </row>
+    <row r="28" spans="1:5">
+      <c r="A28" s="6" t="s">
         <v>27</v>
-      </c>
-      <c r="B27" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="C27" s="5">
-        <v>165.2</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" s="6" t="s">
-        <v>29</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>28</v>
       </c>
       <c r="C28" s="5">
-        <v>103.3</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+        <v>165.2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5">
       <c r="A29" s="6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>28</v>
       </c>
       <c r="C29" s="5">
-        <v>94.6</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+        <v>103.3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5">
       <c r="A30" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>28</v>
       </c>
       <c r="C30" s="5">
-        <v>56.1</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+        <v>94.6</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5">
       <c r="A31" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B31" s="3" t="s">
         <v>28</v>
       </c>
       <c r="C31" s="5">
-        <v>73.3</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+        <v>56.1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5">
       <c r="A32" s="6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B32" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C32" s="18">
-        <v>56.1</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C32" s="5">
+        <v>73.3</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3">
       <c r="A33" s="6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B33" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C33" s="5">
-        <v>91.4</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C33" s="18">
+        <v>56.1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3">
       <c r="A34" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B34" s="3" t="s">
         <v>28</v>
       </c>
       <c r="C34" s="5">
+        <v>91.4</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3">
+      <c r="A35" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C35" s="5">
         <v>146.1</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" s="6" t="s">
+    <row r="36" spans="1:3">
+      <c r="A36" s="6" t="s">
         <v>36</v>
-      </c>
-      <c r="B35" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C35" s="3">
-        <v>0.78</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" s="6" t="s">
-        <v>38</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C36" s="19">
-        <v>2.48</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C36" s="3">
+        <v>0.78</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3">
       <c r="A37" s="6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B37" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C37" s="20">
-        <v>9.4E-2</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C37" s="19">
+        <v>2.48</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3">
       <c r="A38" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B38" s="3" t="s">
         <v>37</v>
@@ -2650,60 +2683,71 @@
         <v>9.4E-2</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3">
       <c r="A39" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B39" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C39" s="5">
+      <c r="C39" s="20">
         <v>9.4E-2</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A40" s="21" t="s">
+    <row r="40" spans="1:3">
+      <c r="A40" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C40" s="5">
+        <v>9.4E-2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3">
+      <c r="A41" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="B40" s="22" t="s">
+      <c r="B41" s="22" t="s">
         <v>37</v>
       </c>
-      <c r="C40" s="23">
+      <c r="C41" s="23">
         <v>9.4E-2</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A41" s="24"/>
-      <c r="B41" s="25"/>
-      <c r="C41" s="24"/>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A42" s="59" t="s">
+    <row r="42" spans="1:3">
+      <c r="A42" s="24"/>
+      <c r="B42" s="25"/>
+      <c r="C42" s="24"/>
+    </row>
+    <row r="43" spans="1:3">
+      <c r="A43" s="63" t="s">
         <v>43</v>
       </c>
-      <c r="B42" s="59"/>
-      <c r="C42" s="59"/>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A43" s="6" t="s">
+      <c r="B43" s="63"/>
+      <c r="C43" s="63"/>
+    </row>
+    <row r="44" spans="1:3">
+      <c r="A44" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="B43" s="3" t="s">
+      <c r="B44" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="C43" s="5">
+      <c r="C44" s="5">
         <v>2019</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="A26:C26"/>
-    <mergeCell ref="A42:C42"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A43:C43"/>
     <mergeCell ref="B2:E2"/>
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="C3:E3"/>
-    <mergeCell ref="C20:D20"/>
     <mergeCell ref="C21:D21"/>
+    <mergeCell ref="C22:D22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -2717,14 +2761,14 @@
     <tabColor rgb="FF595959"/>
   </sheetPr>
   <dimension ref="A1:X34"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="44.7109375" customWidth="1"/>
     <col min="2" max="24" width="14.7109375" customWidth="1"/>
     <col min="25" max="113" width="5.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:24">
       <c r="C1" s="5">
         <v>1995</v>
       </c>
@@ -2792,7 +2836,7 @@
         <v>2016</v>
       </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:24">
       <c r="A2" s="26" t="s">
         <v>46</v>
       </c>
@@ -2866,7 +2910,7 @@
         <v>7442135578</v>
       </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:24">
       <c r="A3" s="8" t="s">
         <v>48</v>
       </c>
@@ -2900,7 +2944,7 @@
       <c r="Q3" s="31"/>
       <c r="R3" s="31"/>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:24">
       <c r="A4" s="26" t="s">
         <v>49</v>
       </c>
@@ -2941,14 +2985,14 @@
       <c r="V4" s="32"/>
       <c r="W4" s="32"/>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:24">
       <c r="A6" s="35" t="s">
         <v>51</v>
       </c>
       <c r="B6" s="36"/>
       <c r="C6" s="37"/>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:24">
       <c r="A7" s="6" t="s">
         <v>52</v>
       </c>
@@ -2959,14 +3003,14 @@
         <v>2500000000</v>
       </c>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:24">
       <c r="A8" s="35" t="s">
         <v>53</v>
       </c>
       <c r="B8" s="36"/>
       <c r="C8" s="37"/>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:24">
       <c r="A9" s="6" t="s">
         <v>54</v>
       </c>
@@ -2977,7 +3021,7 @@
         <v>1526</v>
       </c>
     </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:24">
       <c r="A10" s="38" t="s">
         <v>56</v>
       </c>
@@ -2988,14 +3032,14 @@
         <v>300</v>
       </c>
     </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:24">
       <c r="A11" s="35" t="s">
         <v>57</v>
       </c>
       <c r="B11" s="36"/>
       <c r="C11" s="37"/>
     </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:24">
       <c r="A12" s="38" t="s">
         <v>58</v>
       </c>
@@ -3006,7 +3050,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:24">
       <c r="A13" s="39" t="s">
         <v>60</v>
       </c>
@@ -3017,12 +3061,12 @@
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:24">
       <c r="A14" s="40"/>
       <c r="B14" s="40"/>
       <c r="C14" s="24"/>
     </row>
-    <row r="16" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:24">
       <c r="A16" s="26" t="s">
         <v>63</v>
       </c>
@@ -3033,7 +3077,7 @@
         <v>378.66</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4">
       <c r="A18" s="6" t="s">
         <v>65</v>
       </c>
@@ -3044,14 +3088,14 @@
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="60" t="s">
+    <row r="20" spans="1:4">
+      <c r="A20" s="64" t="s">
         <v>67</v>
       </c>
-      <c r="B20" s="60"/>
-      <c r="C20" s="60"/>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B20" s="64"/>
+      <c r="C20" s="64"/>
+    </row>
+    <row r="21" spans="1:4">
       <c r="A21" s="6" t="s">
         <v>68</v>
       </c>
@@ -3062,7 +3106,7 @@
         <v>43659</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4">
       <c r="A22" s="6" t="s">
         <v>70</v>
       </c>
@@ -3073,10 +3117,10 @@
         <v>7091</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4">
       <c r="A23" s="16"/>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4">
       <c r="A24" t="s">
         <v>71</v>
       </c>
@@ -3084,17 +3128,17 @@
         <v>72</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="60" t="s">
+    <row r="25" spans="1:4">
+      <c r="A25" s="64" t="s">
         <v>73</v>
       </c>
-      <c r="B25" s="60"/>
-      <c r="C25" s="65" t="s">
+      <c r="B25" s="64"/>
+      <c r="C25" s="69" t="s">
         <v>74</v>
       </c>
-      <c r="D25" s="65"/>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D25" s="69"/>
+    </row>
+    <row r="26" spans="1:4">
       <c r="A26" s="6" t="s">
         <v>75</v>
       </c>
@@ -3106,7 +3150,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4">
       <c r="A27" s="6" t="s">
         <v>78</v>
       </c>
@@ -3114,11 +3158,11 @@
         <v>7</v>
       </c>
       <c r="C27" s="5">
-        <v>2.01E-2</v>
+        <v>750</v>
       </c>
       <c r="D27" s="5"/>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4">
       <c r="A28" s="6" t="s">
         <v>79</v>
       </c>
@@ -3126,26 +3170,26 @@
         <v>7</v>
       </c>
       <c r="C28" s="5">
-        <v>2.5</v>
+        <v>50</v>
       </c>
       <c r="D28" s="5"/>
     </row>
-    <row r="31" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" ht="30">
       <c r="A31" s="46" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4">
       <c r="A32" s="41" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:1">
       <c r="A33" s="41" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:1">
       <c r="A34" s="41" t="s">
         <v>83</v>
       </c>
@@ -3167,16 +3211,20 @@
   <sheetPr>
     <tabColor rgb="FF595959"/>
   </sheetPr>
-  <dimension ref="A1:AD43"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AK43"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="44.7109375" customWidth="1"/>
     <col min="2" max="24" width="14.7109375" customWidth="1"/>
     <col min="25" max="26" width="12.140625" customWidth="1"/>
+    <col min="27" max="27" width="12" bestFit="1" customWidth="1"/>
     <col min="28" max="28" width="13" customWidth="1"/>
+    <col min="29" max="33" width="12" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="12" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:37">
       <c r="C1" s="5">
         <v>1995</v>
       </c>
@@ -3243,8 +3291,35 @@
       <c r="X1" s="5">
         <v>2016</v>
       </c>
-    </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="Y1" s="5">
+        <v>2017</v>
+      </c>
+      <c r="Z1" s="5">
+        <v>2018</v>
+      </c>
+      <c r="AA1" s="5">
+        <v>2019</v>
+      </c>
+      <c r="AB1" s="5">
+        <v>2020</v>
+      </c>
+      <c r="AC1" s="5">
+        <v>2021</v>
+      </c>
+      <c r="AD1" s="5">
+        <v>2022</v>
+      </c>
+      <c r="AE1" s="5">
+        <v>2023</v>
+      </c>
+      <c r="AF1" s="5">
+        <v>2024</v>
+      </c>
+      <c r="AG1" s="5">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="2" spans="1:37">
       <c r="A2" s="47" t="s">
         <v>46</v>
       </c>
@@ -3309,34 +3384,43 @@
         <v>441257711</v>
       </c>
       <c r="V2" s="49">
-        <v>442266046</v>
+        <v>442268078</v>
       </c>
       <c r="W2" s="49">
-        <v>442911027</v>
+        <v>442924865</v>
       </c>
       <c r="X2" s="49">
-        <v>443987823</v>
-      </c>
-      <c r="Y2">
-        <v>444655529</v>
-      </c>
-      <c r="Z2">
-        <v>445287011</v>
-      </c>
-      <c r="AA2">
-        <v>446135629</v>
-      </c>
-      <c r="AB2">
-        <v>447015600</v>
-      </c>
-      <c r="AC2">
-        <v>445872542</v>
-      </c>
-      <c r="AD2">
-        <v>445837374</v>
-      </c>
-    </row>
-    <row r="3" spans="1:30" x14ac:dyDescent="0.25">
+        <v>444003268</v>
+      </c>
+      <c r="Y2" s="49">
+        <v>444670605</v>
+      </c>
+      <c r="Z2" s="49">
+        <v>445301376</v>
+      </c>
+      <c r="AA2" s="49">
+        <v>446149924</v>
+      </c>
+      <c r="AB2" s="49">
+        <v>447030024</v>
+      </c>
+      <c r="AC2" s="49">
+        <v>445891011</v>
+      </c>
+      <c r="AD2" s="49">
+        <v>445998928</v>
+      </c>
+      <c r="AE2" s="49">
+        <v>447704445</v>
+      </c>
+      <c r="AF2" s="49">
+        <v>449309618</v>
+      </c>
+      <c r="AG2" s="49">
+        <v>450380320</v>
+      </c>
+    </row>
+    <row r="3" spans="1:37">
       <c r="A3" s="8" t="s">
         <v>48</v>
       </c>
@@ -3378,10 +3462,17 @@
       <c r="T3" s="51"/>
       <c r="U3" s="51"/>
       <c r="V3" s="51"/>
-      <c r="W3" s="51"/>
-      <c r="X3" s="51"/>
-    </row>
-    <row r="4" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="X3" s="59"/>
+      <c r="Z3" s="59"/>
+      <c r="AB3" s="59"/>
+      <c r="AD3" s="59"/>
+      <c r="AF3" s="59"/>
+      <c r="AH3" s="59"/>
+      <c r="AI3" s="58"/>
+      <c r="AJ3" s="59"/>
+      <c r="AK3" s="58"/>
+    </row>
+    <row r="4" spans="1:37">
       <c r="A4" s="26" t="s">
         <v>49</v>
       </c>
@@ -3407,14 +3498,17 @@
         <v>553.37097498222204</v>
       </c>
     </row>
-    <row r="6" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:37">
+      <c r="AC5" s="59"/>
+    </row>
+    <row r="6" spans="1:37">
       <c r="A6" s="35" t="s">
         <v>51</v>
       </c>
       <c r="B6" s="36"/>
       <c r="C6" s="37"/>
     </row>
-    <row r="7" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:37">
       <c r="A7" s="6" t="s">
         <v>52</v>
       </c>
@@ -3425,17 +3519,17 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:37">
       <c r="A8" s="52"/>
       <c r="B8" s="53"/>
       <c r="C8" s="16"/>
     </row>
-    <row r="11" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:37">
       <c r="A11" s="52"/>
       <c r="B11" s="53"/>
       <c r="C11" s="16"/>
     </row>
-    <row r="13" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:37">
       <c r="A13" s="42" t="s">
         <v>61</v>
       </c>
@@ -3527,7 +3621,7 @@
         <v>2120</v>
       </c>
     </row>
-    <row r="14" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:37">
       <c r="A14" s="6" t="s">
         <v>61</v>
       </c>
@@ -3601,7 +3695,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:37">
       <c r="A16" s="26" t="s">
         <v>63</v>
       </c>
@@ -3616,10 +3710,10 @@
       </c>
       <c r="I16" s="58"/>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9">
       <c r="I17" s="58"/>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9">
       <c r="A18" s="6" t="s">
         <v>65</v>
       </c>
@@ -3631,18 +3725,18 @@
       </c>
       <c r="I18" s="58"/>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9">
       <c r="I19" s="58"/>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="60" t="s">
+    <row r="20" spans="1:9">
+      <c r="A20" s="64" t="s">
         <v>67</v>
       </c>
-      <c r="B20" s="60"/>
-      <c r="C20" s="60"/>
+      <c r="B20" s="64"/>
+      <c r="C20" s="64"/>
       <c r="I20" s="58"/>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9">
       <c r="A21" s="6" t="s">
         <v>68</v>
       </c>
@@ -3654,7 +3748,7 @@
       </c>
       <c r="I21" s="58"/>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9">
       <c r="A22" s="6" t="s">
         <v>70</v>
       </c>
@@ -3666,27 +3760,27 @@
       </c>
       <c r="I22" s="58"/>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9">
       <c r="I23" s="58"/>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9">
       <c r="I24" s="58"/>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9">
       <c r="I25" s="58"/>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9">
       <c r="I26" s="58"/>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27" s="60" t="s">
+    <row r="27" spans="1:9">
+      <c r="A27" s="64" t="s">
         <v>85</v>
       </c>
-      <c r="B27" s="60"/>
-      <c r="C27" s="60"/>
+      <c r="B27" s="64"/>
+      <c r="C27" s="64"/>
       <c r="I27" s="58"/>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9">
       <c r="A28" s="6" t="s">
         <v>86</v>
       </c>
@@ -3698,49 +3792,49 @@
       </c>
       <c r="I28" s="58"/>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9">
       <c r="I29" s="58"/>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9">
       <c r="I30" s="58"/>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9">
       <c r="I31" s="58"/>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9">
       <c r="I32" s="58"/>
     </row>
-    <row r="33" spans="9:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="9:9">
       <c r="I33" s="58"/>
     </row>
-    <row r="34" spans="9:9" x14ac:dyDescent="0.25">
+    <row r="34" spans="9:9">
       <c r="I34" s="58"/>
     </row>
-    <row r="35" spans="9:9" x14ac:dyDescent="0.25">
+    <row r="35" spans="9:9">
       <c r="I35" s="58"/>
     </row>
-    <row r="36" spans="9:9" x14ac:dyDescent="0.25">
+    <row r="36" spans="9:9">
       <c r="I36" s="58"/>
     </row>
-    <row r="37" spans="9:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="9:9">
       <c r="I37" s="58"/>
     </row>
-    <row r="38" spans="9:9" x14ac:dyDescent="0.25">
+    <row r="38" spans="9:9">
       <c r="I38" s="58"/>
     </row>
-    <row r="39" spans="9:9" x14ac:dyDescent="0.25">
+    <row r="39" spans="9:9">
       <c r="I39" s="58"/>
     </row>
-    <row r="40" spans="9:9" x14ac:dyDescent="0.25">
+    <row r="40" spans="9:9">
       <c r="I40" s="58"/>
     </row>
-    <row r="41" spans="9:9" x14ac:dyDescent="0.25">
+    <row r="41" spans="9:9">
       <c r="I41" s="58"/>
     </row>
-    <row r="42" spans="9:9" x14ac:dyDescent="0.25">
+    <row r="42" spans="9:9">
       <c r="I42" s="58"/>
     </row>
-    <row r="43" spans="9:9" x14ac:dyDescent="0.25">
+    <row r="43" spans="9:9">
       <c r="I43" s="58"/>
     </row>
   </sheetData>
@@ -3749,8 +3843,8 @@
     <mergeCell ref="A27:C27"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-  <legacyDrawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -3760,7 +3854,7 @@
     <tabColor rgb="FF595959"/>
   </sheetPr>
   <dimension ref="A1:X17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="44.7109375" customWidth="1"/>
     <col min="2" max="24" width="14.7109375" customWidth="1"/>
@@ -3768,7 +3862,7 @@
     <col min="28" max="28" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:24">
       <c r="C1" s="5">
         <v>1995</v>
       </c>
@@ -3836,7 +3930,7 @@
         <v>2016</v>
       </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:24">
       <c r="A2" s="26" t="s">
         <v>46</v>
       </c>
@@ -3910,14 +4004,14 @@
         <v>7448332</v>
       </c>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:24">
       <c r="A4" s="35" t="s">
         <v>51</v>
       </c>
       <c r="B4" s="36"/>
       <c r="C4" s="37"/>
     </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:24">
       <c r="A5" s="6" t="s">
         <v>52</v>
       </c>
@@ -3928,17 +4022,17 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:24">
       <c r="A6" s="52"/>
       <c r="B6" s="53"/>
       <c r="C6" s="16"/>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:24">
       <c r="A7" s="52"/>
       <c r="B7" s="53"/>
       <c r="C7" s="16"/>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:24">
       <c r="A9" s="42" t="s">
         <v>61</v>
       </c>
@@ -4030,7 +4124,7 @@
         <v>2120</v>
       </c>
     </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:24">
       <c r="A10" s="6" t="s">
         <v>61</v>
       </c>
@@ -4104,7 +4198,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:24">
       <c r="A13" s="6" t="s">
         <v>65</v>
       </c>
@@ -4115,14 +4209,14 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A15" s="60" t="s">
+    <row r="15" spans="1:24">
+      <c r="A15" s="64" t="s">
         <v>67</v>
       </c>
-      <c r="B15" s="60"/>
-      <c r="C15" s="60"/>
-    </row>
-    <row r="16" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="B15" s="64"/>
+      <c r="C15" s="64"/>
+    </row>
+    <row r="16" spans="1:24">
       <c r="A16" s="6" t="s">
         <v>68</v>
       </c>
@@ -4133,7 +4227,7 @@
         <v>2.7869999999999999</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3">
       <c r="A17" s="6" t="s">
         <v>70</v>
       </c>

</xml_diff>